<commit_message>
Posters for every film, light and dark themes, projection countdown draw
- Posters: TMDB records found by hand for Chad and Yemen, Films Around the
  World posters for Grenada and Marshall Islands (credited), typographic
  posters for the 9 films with none; build.py accepts a forced tmdb_id
- Light theme alongside the dark one: follows the system, toggle in the
  header, remembered locally, no flash on load
- Random draw: projection leader countdown over the map, then the ticket
  slides out like a dispenser
- French notes: 'No sourced box office data.' translated
</commit_message>
<xml_diff>
--- a/films-du-monde.xlsx
+++ b/films-du-monde.xlsx
@@ -6317,7 +6317,7 @@
       <c r="R71" s="5" t="inlineStr"/>
       <c r="S71" s="5" t="inlineStr">
         <is>
-          <t>Aucune donnée sourcée trouvée dans cette passe</t>
+          <t>Affiche absente de TMDB, reprise de Films Around the World. Aucune donnée sourcée trouvée dans cette passe</t>
         </is>
       </c>
     </row>
@@ -7267,7 +7267,7 @@
       <c r="R83" s="5" t="inlineStr"/>
       <c r="S83" s="5" t="inlineStr">
         <is>
-          <t>No sourced box office data.</t>
+          <t>Affiche absente de TMDB, reprise de Films Around the World. No sourced box office data.</t>
         </is>
       </c>
     </row>
@@ -15123,7 +15123,11 @@
           <t>Bye Bye Africa</t>
         </is>
       </c>
-      <c r="F182" s="3" t="inlineStr"/>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>Bye Bye Africa</t>
+        </is>
+      </c>
       <c r="G182" s="3" t="inlineStr">
         <is>
           <t>1999</t>
@@ -15131,7 +15135,9 @@
       </c>
       <c r="H182" s="3" t="inlineStr"/>
       <c r="I182" s="3" t="inlineStr"/>
-      <c r="J182" s="3" t="inlineStr"/>
+      <c r="J182" s="3" t="n">
+        <v>87</v>
+      </c>
       <c r="K182" s="5" t="inlineStr">
         <is>
           <t>choix « native » de Films Around the World</t>
@@ -15143,7 +15149,11 @@
           <t>https://filmsaroundthe.world/country/chad/films/bye-bye-africa-fb34bc995d48acfbe/</t>
         </is>
       </c>
-      <c r="N182" s="5" t="inlineStr"/>
+      <c r="N182" s="6" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/276186</t>
+        </is>
+      </c>
       <c r="O182" s="5" t="inlineStr"/>
       <c r="P182" s="5" t="inlineStr">
         <is>
@@ -15158,7 +15168,7 @@
       <c r="R182" s="5" t="inlineStr"/>
       <c r="S182" s="5" t="inlineStr">
         <is>
-          <t>pas de box-office national suivi ou publié trouvé</t>
+          <t>Fiche TMDB retrouvée à la main (TMDB date le film de sa sortie française, 2003). pas de box-office national suivi ou publié trouvé</t>
         </is>
       </c>
     </row>
@@ -16393,7 +16403,11 @@
           <t>I'm Nojoum, Age 10 and Divorced</t>
         </is>
       </c>
-      <c r="F198" s="3" t="inlineStr"/>
+      <c r="F198" s="3" t="inlineStr">
+        <is>
+          <t>Moi Nojoom, 10ans et divorcée</t>
+        </is>
+      </c>
       <c r="G198" s="3" t="inlineStr">
         <is>
           <t>2014</t>
@@ -16401,19 +16415,29 @@
       </c>
       <c r="H198" s="3" t="inlineStr"/>
       <c r="I198" s="3" t="inlineStr"/>
-      <c r="J198" s="3" t="inlineStr"/>
+      <c r="J198" s="3" t="n">
+        <v>96</v>
+      </c>
       <c r="K198" s="5" t="inlineStr">
         <is>
           <t>choix « native » de Films Around the World</t>
         </is>
       </c>
-      <c r="L198" s="5" t="inlineStr"/>
+      <c r="L198" s="5" t="inlineStr">
+        <is>
+          <t>location : Apple TV Store, YouTube, Sooner ; achat : YouTube, Canal VOD, Sooner</t>
+        </is>
+      </c>
       <c r="M198" s="6" t="inlineStr">
         <is>
           <t>https://filmsaroundthe.world/country/yemen/films/i-m-nojoum-age-10-and-divorced-f9b86d068ccb9a509/</t>
         </is>
       </c>
-      <c r="N198" s="5" t="inlineStr"/>
+      <c r="N198" s="6" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/341182</t>
+        </is>
+      </c>
       <c r="O198" s="5" t="inlineStr"/>
       <c r="P198" s="5" t="inlineStr">
         <is>
@@ -16428,7 +16452,7 @@
       <c r="R198" s="5" t="inlineStr"/>
       <c r="S198" s="5" t="inlineStr">
         <is>
-          <t>pas de box-office national suivi ou publié trouvé</t>
+          <t>Fiche TMDB retrouvée à la main (titre anglais I Am Nojoom). pas de box-office national suivi ou publié trouvé</t>
         </is>
       </c>
     </row>
@@ -16943,45 +16967,47 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M181" r:id="rId349"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N181" r:id="rId350"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M182" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M183" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N183" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N184" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N185" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N186" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N187" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N188" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N189" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N190" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N191" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N192" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N193" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N194" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N195" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N196" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N197" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N199" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N200" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N182" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M183" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N183" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N184" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N185" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N186" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N187" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N188" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N189" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N190" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M191" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N191" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M192" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N192" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M193" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N193" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M194" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N194" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M195" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N195" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M196" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N196" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M197" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N197" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M198" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N198" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M199" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N199" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M200" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N200" r:id="rId388"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId387"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId389"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>